<commit_message>
docs: add detailed comments to all 34 files (Java, XML, properties) - no code changes
</commit_message>
<xml_diff>
--- a/resources/Youth_beta.xlsx
+++ b/resources/Youth_beta.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Email</t>
   </si>
@@ -54,6 +54,18 @@
   </si>
   <si>
     <t>AdaWindler@yopmail.com</t>
+  </si>
+  <si>
+    <t>JonahBarton@yopmail.com</t>
+  </si>
+  <si>
+    <t>MittieHartmann@yopmail.com</t>
+  </si>
+  <si>
+    <t>ChaunceyStoltenberg@yopmail.com</t>
+  </si>
+  <si>
+    <t>FidelHahn@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1213,52 +1225,72 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1">
-      <c r="A6" t="s">
+      <c r="A6" t="s" s="0">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" t="s">
+      <c r="A7" t="s" s="0">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" t="s">
+      <c r="A8" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" t="s">
+      <c r="A9" t="s" s="0">
         <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>